<commit_message>
[docs] add R6 (CI reported success without running tests) and W3 log entries
</commit_message>
<xml_diff>
--- a/docs/CISC594_Risk_Management_Report_Draft_EComLite.xlsx
+++ b/docs/CISC594_Risk_Management_Report_Draft_EComLite.xlsx
@@ -1077,6 +1077,95 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="158.4" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Build &amp; Verification Pipeline (CI)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>CI reports success without executing any tests</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>The CI workflow (.github/workflows/ci.yml) runs "dotnet test" with no project argument, so it resolves the root solution EComLite.sln. That solution registered only EComLite.Web and omitted EComLite.Tests, so the command matched zero test projects, exited 0, and reported a passing build. Every push and pull request therefore displayed a green check while none of the 34 automated tests actually ran. A regression - including one that breaks the order-status transition rules protecting R4 - could be merged with no signal.</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Min Hsuan Wu</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>1x4</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Likelihood 4: the condition was already active and undetected across multiple merges (CI was added in 61cd86a and PR #1/#2 both merged under a green check). Nothing in the pipeline surfaces an empty test run, so it persists silently until manually inspected.
+[Updated 2026-07-27] Likelihood reduced 4-&gt;1: EComLite.Tests is now registered in EComLite.sln, and a solution-level "dotnet test" (the exact command CI runs) discovers and executes the suite - verified locally with 34 passed / 0 failed. Consequence remains 4 because the pipeline still would not flag a future empty run.</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Consequence 4: the project loses its automated safety net. Mitigations verified only by tests (notably R4 order status transition validation) become unenforced, and the green check actively creates false confidence, which is more damaging than having no CI at all.</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Software Mitigation. Register EComLite.Tests in EComLite.sln so the solution-wide "dotnet test" discovers it. Additionally, treat an empty test run as a failure by asserting a minimum executed-test count, so a silently skipped suite can never present as a pass.
+[Status 2026-07-27] PARTIALLY IMPLEMENTED: EComLite.Tests added to EComLite.sln, so CI now executes all 34 tests. NOT YET IMPLEMENTED: the minimum executed-test-count assertion (FR-6.2.1) that would make an empty test run fail the build.</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>The system's CI pipeline shall execute the full automated test suite on every push and pull request, and shall report success only when all discovered tests have actually run and passed.</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>The CI pipeline shall not report a successful build when zero test projects were discovered or zero tests were executed.</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>If the pipeline discovers no test projects or executes no tests, it shall fail the run and report the empty discovery as the failure reason.</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>FR-6.1.1: SolutionConfiguration shall include every test project so that a solution-level test command discovers the full suite.
+FR-6.1.2: CIWorkflow shall execute the automated test suite on every push and pull request event.</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>FR-6.2.1: CIWorkflow shall reject a run outcome of "success" when the number of executed tests is zero.</t>
+        </is>
+      </c>
+      <c r="R7" s="7" t="inlineStr">
+        <is>
+          <t>FR-6.3.1: CIWorkflow shall fail the job and emit a diagnostic message identifying empty test discovery when no tests are executed.</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
       <c r="C8" s="8" t="n"/>
       <c r="D8" s="8" t="n"/>
@@ -1279,7 +1368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1851,30 +1940,114 @@
       </c>
       <c r="C14" s="22" t="inlineStr">
         <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>Identified (new)</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>4 x 4 = 16</t>
+        </is>
+      </c>
+      <c r="G14" s="23" t="inlineStr">
+        <is>
+          <t>New risk found while preparing to commit the V2 transition tests: CI ran "dotnet test" against EComLite.sln, which omitted EComLite.Tests, so all pushes passed green with zero tests executed. Highest-scoring open risk.</t>
+        </is>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>.github/workflows/ci.yml + EComLite.sln</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>Mitigation implemented</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>4 x 4 = 16</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>1 x 4 = 4</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="inlineStr">
+        <is>
+          <t>EComLite.Tests registered in EComLite.sln; solution-level "dotnet test" now discovers and runs 34 tests (0 failed). Likelihood 4 -&gt; 1; consequence unchanged. Residual: pipeline still would not flag a future empty run.</t>
+        </is>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>Verified locally: 34 passed, 0 failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
         <is>
           <t>No risks retired</t>
         </is>
       </c>
-      <c r="E14" s="22" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F14" s="22" t="inlineStr">
+      <c r="F16" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G14" s="23" t="inlineStr">
-        <is>
-          <t>No risks retired this week. R3 and R4 remain tracked at reduced scores as regression guards even though mitigations are implemented.</t>
-        </is>
-      </c>
-      <c r="H14" s="23" t="inlineStr">
+      <c r="G16" s="23" t="inlineStr">
+        <is>
+          <t>No risks retired this week. R3, R4 and R6 remain tracked at reduced scores as regression guards even though their mitigations are implemented.</t>
+        </is>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
[docs] update risk register: R1/R2 mitigated, R5 partial, add W4 weekly log
</commit_message>
<xml_diff>
--- a/docs/CISC594_Risk_Management_Report_Draft_EComLite.xlsx
+++ b/docs/CISC594_Risk_Management_Report_Draft_EComLite.xlsx
@@ -645,22 +645,23 @@
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>4</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>3x4</t>
+          <t>1x4</t>
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J2" s="7" t="inlineStr">
         <is>
-          <t>Rated 3 (Moderate) because double-submission from double-clicks or slow network retries is a common occurrence in web checkout flows, and the current implementation does not yet enforce an idempotency key across the full checkout request path.</t>
+          <t>Rated 3 (Moderate) because double-submission from double-clicks or slow network retries is a common occurrence in web checkout flows, and the current implementation does not yet enforce an idempotency key across the full checkout request path.
+[Updated 2026-08-02] Likelihood reduced 3-&gt;1: checkout now enforces a unique idempotency key (Order.IdempotencyKey with a filtered unique database index; CheckoutService returns the existing order on a repeat submission). Covered by CheckoutServiceTests.cs. See branch feature/v2-idempotency-cart.</t>
         </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
@@ -674,7 +675,8 @@
 Generate a unique idempotency key per checkout session and require it on the order-creation request.
 Wrap order creation in a database transaction with a unique constraint on (CartId, IdempotencyKey).
 Disable the "Place Order" button immediately after the first click until a response is received.
-This mitigation reduces the likelihood of duplicate orders and lowers the risk from its current score.</t>
+This mitigation reduces the likelihood of duplicate orders and lowers the risk from its current score.
+[Status 2026-08-02] IMPLEMENTED: idempotency key + unique index + CheckoutService.PlaceOrderIdempotentAsync; the Place Order flow reuses one session token per checkout. Automated tests pass. Residual: client-side button-disable and duplicate-attempt audit logging not yet added.</t>
         </is>
       </c>
       <c r="M2" s="7" t="inlineStr">
@@ -738,22 +740,23 @@
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>3</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>4x3</t>
+          <t>1x3</t>
         </is>
       </c>
       <c r="I3" s="4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Rated 4 (High) because checkout can take several minutes when a customer compares shipping options or looks up payment information, and the default ASP.NET Core Identity session/cookie timeout is short relative to that.</t>
+          <t>Rated 4 (High) because checkout can take several minutes when a customer compares shipping options or looks up payment information, and the default ASP.NET Core Identity session/cookie timeout is short relative to that.
+[Updated 2026-08-02] Likelihood reduced 4-&gt;1: the cart is now persisted to the database keyed by user ID (PersistentCartService + PersistedCart table) and restored when the session cart is empty, so it survives session expiry. Covered by PersistentCartServiceTests.cs.</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -766,7 +769,8 @@
           <t>Software Mitigation.
 Persist cart contents to the database keyed by user ID rather than only in the session/cookie, so the cart survives session expiry.
 Use sliding expiration during active checkout.
-Prompt re-authentication without discarding the cart.</t>
+Prompt re-authentication without discarding the cart.
+[Status 2026-08-02] IMPLEMENTED: DB-backed cart keyed by user ID with restore-on-empty in the Cart page. Residual: the re-authentication redirect preserving the return URL relies on the ASP.NET Core Identity default and is not yet covered by an automated browser test.</t>
         </is>
       </c>
       <c r="M3" s="7" t="inlineStr">
@@ -859,7 +863,8 @@
 Enforce [Authorize(Roles="Admin")] at the controller level, not just by hiding UI elements client-side.
 Add automated integration tests asserting HTTP 403 responses for non-admin roles on every admin route.
 Centralize the authorization policy rather than relying on per-action checks.
-[Status 2026-07-25] IMPLEMENTED: [Authorize(Roles="Admin")] enforced at controller level (not UI-only) plus role seeding. Merged in PR #2.</t>
+[Status 2026-07-25] IMPLEMENTED: [Authorize(Roles="Admin")] enforced at controller level (not UI-only) plus role seeding. Merged in PR #2.
+[Note 2026-08-02] Role infrastructure (AddRoles + Admin role seeding) is in place, but the Admin dashboard routes themselves (Version 2 Item 2) are not yet built, so the route-level [Authorize(Roles="Admin")] enforcement and the 403 integration tests will be added and verified when those pages are implemented.</t>
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr">
@@ -1016,22 +1021,23 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>5</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>2x5</t>
+          <t>1x5</t>
         </is>
       </c>
       <c r="I6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>Likelihood 2: seeding currently runs at application startup and is not yet gated by environment, but exploitation still requires the seeding to reach a production database and the default credential to remain unchanged.</t>
+          <t>Likelihood 2: seeding currently runs at application startup and is not yet gated by environment, but exploitation still requires the seeding to reach a production database and the default credential to remain unchanged.
+[Updated 2026-08-02] Likelihood reduced 2-&gt;1: the seeder no longer hardcodes any credential; an admin account is created only when AdminUser:Email/Password are supplied through secure configuration (user-secrets or environment variables), so no default-password account is ever seeded.</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
@@ -1041,7 +1047,8 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>Software Mitigation. Gate role/data seeding behind an explicit environment check (Development/Test only); load the initial admin credential from protected secret/configuration storage instead of source code, and force rotation on first use; never seed a known default password in Production.</t>
+          <t>Software Mitigation. Gate role/data seeding behind an explicit environment check (Development/Test only); load the initial admin credential from protected secret/configuration storage instead of source code, and force rotation on first use; never seed a known default password in Production.
+[Status 2026-08-02] PARTIALLY IMPLEMENTED: admin credential loaded from protected configuration, never from source; no default password seeded (IdentitySeeder). NOT YET IMPLEMENTED: an explicit environment gate that refuses/aborts seeding in Production (FR-5.2.1 / FR-5.3.1).</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
@@ -1368,7 +1375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2053,6 +2060,174 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>Mitigation implemented / Re-scored</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>3 x 4 = 12</t>
+        </is>
+      </c>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>1 x 4 = 4</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="inlineStr">
+        <is>
+          <t>Idempotency key enforced on order creation (Order.IdempotencyKey + filtered unique index; CheckoutService returns the existing order on a repeat submission). Likelihood 3 -&gt; 1.</t>
+        </is>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>feature/v2-idempotency-cart; CheckoutServiceTests.cs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>Mitigation implemented / Re-scored</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>4 x 3 = 12</t>
+        </is>
+      </c>
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>1 x 3 = 3</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>Cart persisted to DB keyed by user ID (PersistentCartService + PersistedCart table), restored when the session cart is empty. Likelihood 4 -&gt; 1.</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>feature/v2-idempotency-cart; PersistentCartServiceTests.cs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Mitigation partially implemented / Re-scored</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="inlineStr">
+        <is>
+          <t>2 x 5 = 10</t>
+        </is>
+      </c>
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>1 x 5 = 5</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="inlineStr">
+        <is>
+          <t>Admin credential now loaded from secure configuration (never from source); no default-password account seeded. Likelihood 2 -&gt; 1. Residual: environment gate to block seeding in Production still pending.</t>
+        </is>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>feature/v2-idempotency-cart; IdentitySeeder.cs</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E20" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t>Automated suite grew to 46 tests (0 failed). R1 and R2 (the two tied top risks) are now mitigated; R5 reduced. Open items: R1/R2 residuals (audit log, browser test) and the R5 production environment gate.</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>test-evidence/2026-07-30-dotnet-test.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>